<commit_message>
tage golden trace FTL match
</commit_message>
<xml_diff>
--- a/programs/assembly/tage_test_trace.xlsx
+++ b/programs/assembly/tage_test_trace.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emerald\zaqal\programs\assembly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F281E1E4-7DA8-4357-8615-65F0E7F1264A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C6D24C-DBCF-43AD-A9F4-4BC21CA979FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28965" yWindow="-2070" windowWidth="11325" windowHeight="25140" xr2:uid="{E346031A-6FE0-420F-941A-72680D802F2C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E346031A-6FE0-420F-941A-72680D802F2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="108">
   <si>
     <t>order</t>
   </si>
@@ -358,6 +358,9 @@
   </si>
   <si>
     <t>PRE GHR</t>
+  </si>
+  <si>
+    <t>Post GHR</t>
   </si>
 </sst>
 </file>
@@ -862,7 +865,9 @@
       <c r="S1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="T1" s="5"/>
+      <c r="T1" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="U1" s="5" t="s">
         <v>68</v>
       </c>
@@ -1458,7 +1463,9 @@
       <c r="S15" s="1">
         <v>0</v>
       </c>
-      <c r="T15" s="1"/>
+      <c r="T15" s="1">
+        <v>1</v>
+      </c>
       <c r="U15" s="1" t="s">
         <v>74</v>
       </c>
@@ -1576,7 +1583,9 @@
       <c r="S18" s="1">
         <v>1</v>
       </c>
-      <c r="T18" s="1"/>
+      <c r="T18" s="1">
+        <v>3</v>
+      </c>
       <c r="U18" s="1" t="s">
         <v>75</v>
       </c>
@@ -1905,7 +1914,9 @@
       <c r="S27" s="1">
         <v>3</v>
       </c>
-      <c r="T27" s="1"/>
+      <c r="T27" s="1">
+        <v>7</v>
+      </c>
       <c r="U27" s="1" t="s">
         <v>76</v>
       </c>
@@ -2076,7 +2087,9 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
+      <c r="G31" s="1">
+        <v>121</v>
+      </c>
       <c r="H31" s="4" t="s">
         <v>73</v>
       </c>
@@ -2104,7 +2117,9 @@
       <c r="R31" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="S31" s="1"/>
+      <c r="S31" s="1">
+        <v>7</v>
+      </c>
       <c r="T31" s="1"/>
       <c r="U31" s="4" t="s">
         <v>77</v>

</xml_diff>